<commit_message>
EmialTextToPay-changes in state from SC to South Carolina
</commit_message>
<xml_diff>
--- a/KatalonData/EmailTextToPay/BillFileLookUp.xlsx
+++ b/KatalonData/EmailTextToPay/BillFileLookUp.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t470258\Documents\VPS-Katalon\KatalonData\EmailTextToPay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{146A62CC-B87A-4D94-B59E-76889275F33D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr documentId="13_ncr:1_{146A62CC-B87A-4D94-B59E-76889275F33D}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{A171AD99-6CB3-481A-968B-971B4AF2105E}"/>
+    <workbookView activeTab="1" windowHeight="11500" windowWidth="19420" xWindow="-110" xr2:uid="{A171AD99-6CB3-481A-968B-971B4AF2105E}" yWindow="-110"/>
   </bookViews>
   <sheets>
-    <sheet name="BFLU" sheetId="1" r:id="rId1"/>
-    <sheet name="BFLUError" sheetId="2" r:id="rId2"/>
+    <sheet name="BFLU" r:id="rId1" sheetId="1"/>
+    <sheet name="BFLUError" r:id="rId2" sheetId="2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="131">
   <si>
     <t>Result</t>
   </si>
@@ -327,12 +327,118 @@
   </si>
   <si>
     <t>Thu Feb 05 00:45:35 IST 2026</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:51:15 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:51:53 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:52:30 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:53:00 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:53:34 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:54:12 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:54:44 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:55:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:55:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:56:21 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:56:53 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:57:26 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:58:00 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:58:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:59:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 11:59:33 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:00:06 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:00:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:01:25 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:01:56 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:02:24 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:03:01 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:03:30 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:06:22 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:07:03 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:07:32 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:08:11 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:08:42 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:09:16 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:09:46 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:10:20 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:10:49 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:11:18 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Feb 17 12:11:49 IST 2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -391,42 +497,42 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
+    <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="49" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf applyFont="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf applyAlignment="1" applyBorder="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="0" numFmtId="49" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1" borderId="1" fillId="0" fontId="3" numFmtId="49" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf applyAlignment="1" applyFont="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf applyAlignment="1" applyFont="1" borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf applyFont="1" borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle builtinId="0" name="Normal" xfId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -443,10 +549,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -481,7 +587,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin panose="02110004020202020204" typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -533,7 +639,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin panose="02110004020202020204" typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -644,21 +750,21 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="12700">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="19050">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cap="flat" cmpd="sng" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -675,7 +781,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw algn="ctr" blurRad="57150" dir="5400000" dist="19050" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -747,27 +853,27 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" name="Office Theme" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F033DD18-DD0F-43E3-A2D0-6223D1731E2C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F033DD18-DD0F-43E3-A2D0-6223D1731E2C}">
   <dimension ref="A1:L24"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.36328125" customWidth="1" collapsed="1"/>
-    <col min="2" max="2" width="26.54296875" customWidth="1" collapsed="1"/>
-    <col min="3" max="3" width="35.453125" customWidth="1" collapsed="1"/>
-    <col min="5" max="5" width="18.7265625" customWidth="1" collapsed="1"/>
-    <col min="6" max="6" width="9.453125" customWidth="1" collapsed="1"/>
-    <col min="7" max="7" width="10.6328125" customWidth="1" collapsed="1"/>
-    <col min="8" max="8" width="26.54296875" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="9" max="9" width="7.6328125" customWidth="1" collapsed="1"/>
-    <col min="11" max="11" width="7.6328125" customWidth="1" collapsed="1"/>
-    <col min="12" max="12" width="27.90625" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="1" max="1" customWidth="true" width="6.36328125" collapsed="true"/>
+    <col min="2" max="2" customWidth="true" width="26.54296875" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" width="35.453125" collapsed="true"/>
+    <col min="5" max="5" customWidth="true" width="18.7265625" collapsed="true"/>
+    <col min="6" max="6" customWidth="true" width="9.453125" collapsed="true"/>
+    <col min="7" max="7" customWidth="true" width="10.6328125" collapsed="true"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="26.54296875" collapsed="true"/>
+    <col min="9" max="9" customWidth="true" width="7.6328125" collapsed="true"/>
+    <col min="11" max="11" customWidth="true" width="7.6328125" collapsed="true"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="27.90625" collapsed="true"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -805,12 +911,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>52</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>97</v>
       </c>
       <c r="C2" t="s">
         <v>17</v>
@@ -825,12 +931,12 @@
         <v>50020006</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="C3" t="s">
         <v>18</v>
@@ -845,12 +951,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="C4" t="s">
         <v>19</v>
@@ -865,12 +971,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>52</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C5" t="s">
         <v>20</v>
@@ -885,12 +991,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>52</v>
       </c>
       <c r="B6" t="s">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="C6" t="s">
         <v>21</v>
@@ -905,12 +1011,12 @@
         <v>282719</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>52</v>
       </c>
       <c r="B7" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="C7" t="s">
         <v>32</v>
@@ -925,12 +1031,12 @@
         <v>884777</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>52</v>
       </c>
       <c r="B8" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="C8" t="s">
         <v>33</v>
@@ -945,12 +1051,12 @@
         <v>915029</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>52</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>104</v>
       </c>
       <c r="C9" t="s">
         <v>22</v>
@@ -968,12 +1074,12 @@
         <v>884777</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>52</v>
       </c>
       <c r="B10" t="s">
-        <v>78</v>
+        <v>105</v>
       </c>
       <c r="C10" t="s">
         <v>23</v>
@@ -991,12 +1097,12 @@
         <v>915029</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>52</v>
       </c>
       <c r="B11" t="s">
-        <v>79</v>
+        <v>106</v>
       </c>
       <c r="C11" t="s">
         <v>24</v>
@@ -1014,12 +1120,12 @@
         <v>915029</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="25.5" x14ac:dyDescent="0.3">
+    <row ht="25.5" r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>52</v>
       </c>
       <c r="B12" t="s">
-        <v>64</v>
+        <v>107</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>25</v>
@@ -1040,12 +1146,12 @@
         <v>915029</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>52</v>
       </c>
       <c r="B13" t="s">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="C13" t="s">
         <v>16</v>
@@ -1075,12 +1181,12 @@
         <v>915029</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>52</v>
       </c>
       <c r="B14" t="s">
-        <v>66</v>
+        <v>109</v>
       </c>
       <c r="C14" t="s">
         <v>28</v>
@@ -1098,12 +1204,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>52</v>
       </c>
       <c r="B15" t="s">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="C15" t="s">
         <v>26</v>
@@ -1121,12 +1227,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="25.5" x14ac:dyDescent="0.3">
+    <row ht="25.5" r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>52</v>
       </c>
       <c r="B16" t="s">
-        <v>81</v>
+        <v>111</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>27</v>
@@ -1144,12 +1250,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>52</v>
       </c>
       <c r="B17" t="s">
-        <v>82</v>
+        <v>112</v>
       </c>
       <c r="C17" t="s">
         <v>29</v>
@@ -1167,12 +1273,12 @@
         <v>282719</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>52</v>
       </c>
       <c r="B18" t="s">
-        <v>83</v>
+        <v>113</v>
       </c>
       <c r="C18" t="s">
         <v>30</v>
@@ -1190,12 +1296,12 @@
         <v>884777</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>52</v>
       </c>
       <c r="B19" t="s">
-        <v>84</v>
+        <v>114</v>
       </c>
       <c r="C19" t="s">
         <v>31</v>
@@ -1213,12 +1319,12 @@
         <v>915029</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>52</v>
       </c>
       <c r="B20" t="s">
-        <v>85</v>
+        <v>115</v>
       </c>
       <c r="C20" t="s">
         <v>34</v>
@@ -1236,12 +1342,12 @@
         <v>282719</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>52</v>
       </c>
       <c r="B21" t="s">
-        <v>86</v>
+        <v>116</v>
       </c>
       <c r="C21" t="s">
         <v>35</v>
@@ -1259,12 +1365,12 @@
         <v>884777</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>52</v>
       </c>
       <c r="B22" t="s">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="C22" t="s">
         <v>36</v>
@@ -1282,12 +1388,12 @@
         <v>915029</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>52</v>
       </c>
       <c r="B23" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="C23" t="s">
         <v>37</v>
@@ -1305,12 +1411,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="13" x14ac:dyDescent="0.3">
+    <row ht="13" r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>52</v>
       </c>
       <c r="B24" t="s">
-        <v>89</v>
+        <v>119</v>
       </c>
       <c r="C24" t="s">
         <v>38</v>
@@ -1330,32 +1436,32 @@
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35650B67-EEEE-43A0-9B0F-50672085E657}">
-  <dimension ref="A1:L12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35650B67-EEEE-43A0-9B0F-50672085E657}">
+  <dimension ref="A1:M12"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.08984375" style="6" customWidth="1" collapsed="1"/>
-    <col min="2" max="2" width="10.36328125" style="8" customWidth="1" collapsed="1"/>
-    <col min="3" max="3" width="24.08984375" style="9" customWidth="1" collapsed="1"/>
-    <col min="4" max="4" width="7.81640625" style="6" customWidth="1" collapsed="1"/>
-    <col min="5" max="5" width="18.453125" style="6" customWidth="1" collapsed="1"/>
-    <col min="6" max="6" width="6.6328125" style="6" customWidth="1" collapsed="1"/>
-    <col min="7" max="7" width="9.81640625" style="6" customWidth="1" collapsed="1"/>
-    <col min="8" max="8" width="15.54296875" style="6" customWidth="1" collapsed="1"/>
-    <col min="9" max="9" width="7.26953125" style="6" customWidth="1" collapsed="1"/>
-    <col min="10" max="10" width="6.6328125" style="6" customWidth="1" collapsed="1"/>
-    <col min="11" max="11" width="6.90625" style="6" customWidth="1" collapsed="1"/>
-    <col min="12" max="12" width="45.1796875" style="8" customWidth="1" collapsed="1"/>
-    <col min="13" max="16384" width="8.7265625" style="6" collapsed="1"/>
+    <col min="1" max="1" customWidth="true" style="6" width="6.08984375" collapsed="true"/>
+    <col min="2" max="2" customWidth="true" style="8" width="10.36328125" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" style="9" width="24.08984375" collapsed="true"/>
+    <col min="4" max="4" customWidth="true" style="6" width="7.81640625" collapsed="true"/>
+    <col min="5" max="5" customWidth="true" style="6" width="18.453125" collapsed="true"/>
+    <col min="6" max="6" customWidth="true" style="6" width="6.6328125" collapsed="true"/>
+    <col min="7" max="7" customWidth="true" style="6" width="9.81640625" collapsed="true"/>
+    <col min="8" max="8" customWidth="true" style="6" width="15.54296875" collapsed="true"/>
+    <col min="9" max="9" customWidth="true" style="6" width="7.26953125" collapsed="true"/>
+    <col min="10" max="10" customWidth="true" style="6" width="6.6328125" collapsed="true"/>
+    <col min="11" max="11" customWidth="true" style="6" width="6.90625" collapsed="true"/>
+    <col min="12" max="12" customWidth="true" style="8" width="45.1796875" collapsed="true"/>
+    <col min="13" max="16384" style="6" width="8.7265625" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1393,12 +1499,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>67</v>
+      <c r="B2" t="s">
+        <v>120</v>
       </c>
       <c r="C2" s="9" t="s">
         <v>41</v>
@@ -1416,12 +1522,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>52</v>
       </c>
-      <c r="B3" s="10" t="s">
-        <v>68</v>
+      <c r="B3" t="s">
+        <v>121</v>
       </c>
       <c r="C3" s="9" t="s">
         <v>42</v>
@@ -1439,12 +1545,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>52</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>69</v>
+      <c r="B4" t="s">
+        <v>122</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>43</v>
@@ -1462,12 +1568,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>52</v>
       </c>
       <c r="B5" t="s">
-        <v>91</v>
+        <v>123</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>44</v>
@@ -1485,12 +1591,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>70</v>
+      <c r="B6" t="s">
+        <v>124</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>45</v>
@@ -1508,12 +1614,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>52</v>
       </c>
       <c r="B7" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>46</v>
@@ -1531,12 +1637,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>52</v>
       </c>
       <c r="B8" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>47</v>
@@ -1554,12 +1660,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="37.5" x14ac:dyDescent="0.25">
+    <row ht="37.5" r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>71</v>
+      <c r="B9" t="s">
+        <v>127</v>
       </c>
       <c r="C9" s="9" t="s">
         <v>48</v>
@@ -1580,12 +1686,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="25" x14ac:dyDescent="0.25">
+    <row ht="25" r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>52</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>72</v>
+      <c r="B10" t="s">
+        <v>128</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>49</v>
@@ -1606,12 +1712,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="37.5" x14ac:dyDescent="0.25">
+    <row ht="37.5" r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>52</v>
       </c>
       <c r="B11" t="s">
-        <v>94</v>
+        <v>129</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>50</v>
@@ -1632,12 +1738,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="37.5" x14ac:dyDescent="0.25">
+    <row ht="37.5" r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>52</v>
       </c>
       <c r="B12" t="s">
-        <v>95</v>
+        <v>130</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>51</v>
@@ -1659,7 +1765,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Due Date Validation for EmailTextToPay-latest
</commit_message>
<xml_diff>
--- a/KatalonData/EmailTextToPay/BillFileLookUp.xlsx
+++ b/KatalonData/EmailTextToPay/BillFileLookUp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t470258\Documents\VPS-Katalon\KatalonData\EmailTextToPay\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69211089-82A4-49BA-8ABF-994FAC3903E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DAC9DAD-98AD-4914-90B7-E2BB443F241E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{A171AD99-6CB3-481A-968B-971B4AF2105E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A171AD99-6CB3-481A-968B-971B4AF2105E}"/>
   </bookViews>
   <sheets>
     <sheet name="BFLU" sheetId="1" r:id="rId1"/>
@@ -1340,7 +1340,7 @@
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.08984375" style="6" customWidth="1" collapsed="1"/>
-    <col min="2" max="2" width="10.36328125" style="8" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="12.08984375" style="8" customWidth="1" collapsed="1"/>
     <col min="3" max="3" width="24.08984375" style="9" customWidth="1" collapsed="1"/>
     <col min="4" max="4" width="7.81640625" style="6" customWidth="1" collapsed="1"/>
     <col min="5" max="5" width="18.453125" style="6" customWidth="1" collapsed="1"/>

</xml_diff>